<commit_message>
data: regenerate unedited review copies with review columns
</commit_message>
<xml_diff>
--- a/data/raw/Democracy in Action/review/dia_2008_organizations_review.xlsx
+++ b/data/raw/Democracy in Action/review/dia_2008_organizations_review.xlsx
@@ -9,17 +9,23 @@
     <sheet name="review" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'review'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'review'!$A$1:$S$16</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t xml:space="preserve">row_id</t>
   </si>
   <si>
+    <t xml:space="preserve">review_action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">review_note</t>
+  </si>
+  <si>
     <t xml:space="preserve">contest_id</t>
   </si>
   <si>
@@ -69,6 +75,9 @@
   </si>
   <si>
     <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">2008D</t>
@@ -678,22 +687,24 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="8.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="40.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="23.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="21.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="8.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="10.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="16.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="8.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="18.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="18.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="40.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="11.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="80.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="8.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="8.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="12.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="40.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="23.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="21.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="8.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="10.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="16.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="18.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="18.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="40.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="11.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="80.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -748,622 +759,718 @@
       <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
+        <v>24</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J2" s="1"/>
-      <c r="K2" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="K2" s="1"/>
       <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="N2" s="1"/>
-      <c r="O2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
       <c r="Q2" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>32</v>
+      <c r="S3" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+        <v>24</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J4" s="1"/>
-      <c r="K4" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="K4" s="1"/>
       <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
+      <c r="M4" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>36</v>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
+        <v>24</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J5" s="1"/>
-      <c r="K5" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="M5" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="N5" s="1"/>
-      <c r="O5" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
       <c r="Q5" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
+        <v>24</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J6" s="1"/>
-      <c r="K6" s="1" t="s">
-        <v>44</v>
-      </c>
+      <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
+      <c r="M6" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="N6" s="1"/>
-      <c r="O6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
       <c r="Q6" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J7" s="1"/>
-      <c r="K7" s="1" t="s">
-        <v>50</v>
-      </c>
+      <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
+      <c r="M7" s="1" t="s">
+        <v>53</v>
+      </c>
       <c r="N7" s="1"/>
-      <c r="O7" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
       <c r="Q7" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J8" s="1"/>
-      <c r="K8" s="1" t="s">
-        <v>56</v>
-      </c>
+      <c r="K8" s="1"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
+      <c r="M8" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="N8" s="1"/>
-      <c r="O8" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
       <c r="Q8" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J9" s="1"/>
-      <c r="K9" s="1" t="s">
-        <v>61</v>
-      </c>
+      <c r="K9" s="1"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
+      <c r="M9" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="N9" s="1"/>
-      <c r="O9" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
       <c r="Q9" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J10" s="1"/>
-      <c r="K10" s="1" t="s">
-        <v>66</v>
-      </c>
+      <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
+      <c r="M10" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="N10" s="1"/>
-      <c r="O10" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
       <c r="Q10" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J11" s="1"/>
-      <c r="K11" s="1" t="s">
-        <v>71</v>
-      </c>
+      <c r="K11" s="1"/>
       <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
+      <c r="M11" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="N11" s="1"/>
-      <c r="O11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
       <c r="Q11" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J12" s="1"/>
-      <c r="K12" s="1" t="s">
-        <v>76</v>
-      </c>
+      <c r="K12" s="1"/>
       <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
+      <c r="M12" s="1" t="s">
+        <v>79</v>
+      </c>
       <c r="N12" s="1"/>
-      <c r="O12" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
       <c r="Q12" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
+        <v>85</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J13" s="1"/>
-      <c r="K13" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
       <c r="Q13" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S13" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
+        <v>92</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J14" s="1"/>
-      <c r="K14" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="K14" s="1"/>
       <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
+      <c r="M14" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="N14" s="1"/>
-      <c r="O14" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
       <c r="Q14" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
+        <v>98</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J15" s="1"/>
-      <c r="K15" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
       <c r="Q15" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S15" s="1" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>101</v>
+        <v>22</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
+        <v>104</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J16" s="1"/>
-      <c r="K16" s="1" t="s">
-        <v>103</v>
-      </c>
+      <c r="K16" s="1"/>
       <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
+      <c r="M16" s="1" t="s">
+        <v>106</v>
+      </c>
       <c r="N16" s="1"/>
-      <c r="O16" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
       <c r="Q16" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S16" s="1" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="17">
@@ -1384,6 +1491,8 @@
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
     </row>
     <row r="18">
       <c r="A18" s="1"/>
@@ -1403,6 +1512,8 @@
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
     </row>
     <row r="19">
       <c r="A19" s="1"/>
@@ -1422,6 +1533,8 @@
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="1"/>
@@ -1441,6 +1554,8 @@
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
     </row>
     <row r="21">
       <c r="A21" s="1"/>
@@ -1460,6 +1575,8 @@
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
+      <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="1"/>
@@ -1479,6 +1596,8 @@
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="1"/>
@@ -1498,6 +1617,8 @@
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="1"/>
@@ -1517,6 +1638,8 @@
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
     </row>
     <row r="25">
       <c r="A25" s="1"/>
@@ -1536,6 +1659,8 @@
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
     </row>
     <row r="26">
       <c r="A26" s="1"/>
@@ -1555,6 +1680,8 @@
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="1"/>
@@ -1574,6 +1701,8 @@
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="1"/>
@@ -1593,6 +1722,8 @@
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="1"/>
@@ -1612,6 +1743,8 @@
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
     </row>
     <row r="30">
       <c r="A30" s="1"/>
@@ -1631,6 +1764,8 @@
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="1"/>
@@ -1650,6 +1785,8 @@
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
     </row>
     <row r="32">
       <c r="A32" s="1"/>
@@ -1669,6 +1806,8 @@
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
     </row>
     <row r="33">
       <c r="A33" s="1"/>
@@ -1688,6 +1827,8 @@
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
     </row>
     <row r="34">
       <c r="A34" s="1"/>
@@ -1707,6 +1848,8 @@
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
     </row>
     <row r="35">
       <c r="A35" s="1"/>
@@ -1726,6 +1869,8 @@
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
+      <c r="S35" s="1"/>
     </row>
     <row r="36">
       <c r="A36" s="1"/>
@@ -1745,6 +1890,8 @@
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
+      <c r="R36" s="1"/>
+      <c r="S36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" s="1"/>
@@ -1764,6 +1911,8 @@
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
+      <c r="R37" s="1"/>
+      <c r="S37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" s="1"/>
@@ -1783,6 +1932,8 @@
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
       <c r="Q38" s="1"/>
+      <c r="R38" s="1"/>
+      <c r="S38" s="1"/>
     </row>
     <row r="39">
       <c r="A39" s="1"/>
@@ -1802,6 +1953,8 @@
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
+      <c r="R39" s="1"/>
+      <c r="S39" s="1"/>
     </row>
     <row r="40">
       <c r="A40" s="1"/>
@@ -1821,6 +1974,8 @@
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
+      <c r="R40" s="1"/>
+      <c r="S40" s="1"/>
     </row>
     <row r="41">
       <c r="A41" s="1"/>
@@ -1840,6 +1995,8 @@
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
       <c r="Q41" s="1"/>
+      <c r="R41" s="1"/>
+      <c r="S41" s="1"/>
     </row>
     <row r="42">
       <c r="A42" s="1"/>
@@ -1859,6 +2016,8 @@
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
+      <c r="R42" s="1"/>
+      <c r="S42" s="1"/>
     </row>
     <row r="43">
       <c r="A43" s="1"/>
@@ -1878,6 +2037,8 @@
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
+      <c r="R43" s="1"/>
+      <c r="S43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="1"/>
@@ -1897,6 +2058,8 @@
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
+      <c r="R44" s="1"/>
+      <c r="S44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="1"/>
@@ -1916,6 +2079,8 @@
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
+      <c r="R45" s="1"/>
+      <c r="S45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="1"/>
@@ -1935,6 +2100,8 @@
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
+      <c r="R46" s="1"/>
+      <c r="S46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="1"/>
@@ -1954,6 +2121,8 @@
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
+      <c r="R47" s="1"/>
+      <c r="S47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="1"/>
@@ -1973,6 +2142,8 @@
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
+      <c r="R48" s="1"/>
+      <c r="S48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="1"/>
@@ -1992,6 +2163,8 @@
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
+      <c r="R49" s="1"/>
+      <c r="S49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="1"/>
@@ -2011,6 +2184,8 @@
       <c r="O50" s="1"/>
       <c r="P50" s="1"/>
       <c r="Q50" s="1"/>
+      <c r="R50" s="1"/>
+      <c r="S50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="1"/>
@@ -2030,6 +2205,8 @@
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
+      <c r="R51" s="1"/>
+      <c r="S51" s="1"/>
     </row>
     <row r="52">
       <c r="A52" s="1"/>
@@ -2049,6 +2226,8 @@
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
       <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
     </row>
     <row r="53">
       <c r="A53" s="1"/>
@@ -2068,6 +2247,8 @@
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
+      <c r="R53" s="1"/>
+      <c r="S53" s="1"/>
     </row>
     <row r="54">
       <c r="A54" s="1"/>
@@ -2087,6 +2268,8 @@
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
+      <c r="R54" s="1"/>
+      <c r="S54" s="1"/>
     </row>
     <row r="55">
       <c r="A55" s="1"/>
@@ -2106,6 +2289,8 @@
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
       <c r="Q55" s="1"/>
+      <c r="R55" s="1"/>
+      <c r="S55" s="1"/>
     </row>
     <row r="56">
       <c r="A56" s="1"/>
@@ -2125,6 +2310,8 @@
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
       <c r="Q56" s="1"/>
+      <c r="R56" s="1"/>
+      <c r="S56" s="1"/>
     </row>
     <row r="57">
       <c r="A57" s="1"/>
@@ -2144,6 +2331,8 @@
       <c r="O57" s="1"/>
       <c r="P57" s="1"/>
       <c r="Q57" s="1"/>
+      <c r="R57" s="1"/>
+      <c r="S57" s="1"/>
     </row>
     <row r="58">
       <c r="A58" s="1"/>
@@ -2163,6 +2352,8 @@
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
       <c r="Q58" s="1"/>
+      <c r="R58" s="1"/>
+      <c r="S58" s="1"/>
     </row>
     <row r="59">
       <c r="A59" s="1"/>
@@ -2182,6 +2373,8 @@
       <c r="O59" s="1"/>
       <c r="P59" s="1"/>
       <c r="Q59" s="1"/>
+      <c r="R59" s="1"/>
+      <c r="S59" s="1"/>
     </row>
     <row r="60">
       <c r="A60" s="1"/>
@@ -2201,6 +2394,8 @@
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
       <c r="Q60" s="1"/>
+      <c r="R60" s="1"/>
+      <c r="S60" s="1"/>
     </row>
     <row r="61">
       <c r="A61" s="1"/>
@@ -2220,6 +2415,8 @@
       <c r="O61" s="1"/>
       <c r="P61" s="1"/>
       <c r="Q61" s="1"/>
+      <c r="R61" s="1"/>
+      <c r="S61" s="1"/>
     </row>
     <row r="62">
       <c r="A62" s="1"/>
@@ -2239,6 +2436,8 @@
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
       <c r="Q62" s="1"/>
+      <c r="R62" s="1"/>
+      <c r="S62" s="1"/>
     </row>
     <row r="63">
       <c r="A63" s="1"/>
@@ -2258,6 +2457,8 @@
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
       <c r="Q63" s="1"/>
+      <c r="R63" s="1"/>
+      <c r="S63" s="1"/>
     </row>
     <row r="64">
       <c r="A64" s="1"/>
@@ -2277,6 +2478,8 @@
       <c r="O64" s="1"/>
       <c r="P64" s="1"/>
       <c r="Q64" s="1"/>
+      <c r="R64" s="1"/>
+      <c r="S64" s="1"/>
     </row>
     <row r="65">
       <c r="A65" s="1"/>
@@ -2296,6 +2499,8 @@
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
       <c r="Q65" s="1"/>
+      <c r="R65" s="1"/>
+      <c r="S65" s="1"/>
     </row>
     <row r="66">
       <c r="A66" s="1"/>
@@ -2315,6 +2520,8 @@
       <c r="O66" s="1"/>
       <c r="P66" s="1"/>
       <c r="Q66" s="1"/>
+      <c r="R66" s="1"/>
+      <c r="S66" s="1"/>
     </row>
     <row r="67">
       <c r="A67" s="1"/>
@@ -2334,6 +2541,8 @@
       <c r="O67" s="1"/>
       <c r="P67" s="1"/>
       <c r="Q67" s="1"/>
+      <c r="R67" s="1"/>
+      <c r="S67" s="1"/>
     </row>
     <row r="68">
       <c r="A68" s="1"/>
@@ -2353,6 +2562,8 @@
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
       <c r="Q68" s="1"/>
+      <c r="R68" s="1"/>
+      <c r="S68" s="1"/>
     </row>
     <row r="69">
       <c r="A69" s="1"/>
@@ -2372,6 +2583,8 @@
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
       <c r="Q69" s="1"/>
+      <c r="R69" s="1"/>
+      <c r="S69" s="1"/>
     </row>
     <row r="70">
       <c r="A70" s="1"/>
@@ -2391,6 +2604,8 @@
       <c r="O70" s="1"/>
       <c r="P70" s="1"/>
       <c r="Q70" s="1"/>
+      <c r="R70" s="1"/>
+      <c r="S70" s="1"/>
     </row>
     <row r="71">
       <c r="A71" s="1"/>
@@ -2410,6 +2625,8 @@
       <c r="O71" s="1"/>
       <c r="P71" s="1"/>
       <c r="Q71" s="1"/>
+      <c r="R71" s="1"/>
+      <c r="S71" s="1"/>
     </row>
     <row r="72">
       <c r="A72" s="1"/>
@@ -2429,6 +2646,8 @@
       <c r="O72" s="1"/>
       <c r="P72" s="1"/>
       <c r="Q72" s="1"/>
+      <c r="R72" s="1"/>
+      <c r="S72" s="1"/>
     </row>
     <row r="73">
       <c r="A73" s="1"/>
@@ -2448,6 +2667,8 @@
       <c r="O73" s="1"/>
       <c r="P73" s="1"/>
       <c r="Q73" s="1"/>
+      <c r="R73" s="1"/>
+      <c r="S73" s="1"/>
     </row>
     <row r="74">
       <c r="A74" s="1"/>
@@ -2467,6 +2688,8 @@
       <c r="O74" s="1"/>
       <c r="P74" s="1"/>
       <c r="Q74" s="1"/>
+      <c r="R74" s="1"/>
+      <c r="S74" s="1"/>
     </row>
     <row r="75">
       <c r="A75" s="1"/>
@@ -2486,6 +2709,8 @@
       <c r="O75" s="1"/>
       <c r="P75" s="1"/>
       <c r="Q75" s="1"/>
+      <c r="R75" s="1"/>
+      <c r="S75" s="1"/>
     </row>
     <row r="76">
       <c r="A76" s="1"/>
@@ -2505,6 +2730,8 @@
       <c r="O76" s="1"/>
       <c r="P76" s="1"/>
       <c r="Q76" s="1"/>
+      <c r="R76" s="1"/>
+      <c r="S76" s="1"/>
     </row>
     <row r="77">
       <c r="A77" s="1"/>
@@ -2524,6 +2751,8 @@
       <c r="O77" s="1"/>
       <c r="P77" s="1"/>
       <c r="Q77" s="1"/>
+      <c r="R77" s="1"/>
+      <c r="S77" s="1"/>
     </row>
     <row r="78">
       <c r="A78" s="1"/>
@@ -2543,6 +2772,8 @@
       <c r="O78" s="1"/>
       <c r="P78" s="1"/>
       <c r="Q78" s="1"/>
+      <c r="R78" s="1"/>
+      <c r="S78" s="1"/>
     </row>
     <row r="79">
       <c r="A79" s="1"/>
@@ -2562,6 +2793,8 @@
       <c r="O79" s="1"/>
       <c r="P79" s="1"/>
       <c r="Q79" s="1"/>
+      <c r="R79" s="1"/>
+      <c r="S79" s="1"/>
     </row>
     <row r="80">
       <c r="A80" s="1"/>
@@ -2581,6 +2814,8 @@
       <c r="O80" s="1"/>
       <c r="P80" s="1"/>
       <c r="Q80" s="1"/>
+      <c r="R80" s="1"/>
+      <c r="S80" s="1"/>
     </row>
     <row r="81">
       <c r="A81" s="1"/>
@@ -2600,6 +2835,8 @@
       <c r="O81" s="1"/>
       <c r="P81" s="1"/>
       <c r="Q81" s="1"/>
+      <c r="R81" s="1"/>
+      <c r="S81" s="1"/>
     </row>
     <row r="82">
       <c r="A82" s="1"/>
@@ -2619,6 +2856,8 @@
       <c r="O82" s="1"/>
       <c r="P82" s="1"/>
       <c r="Q82" s="1"/>
+      <c r="R82" s="1"/>
+      <c r="S82" s="1"/>
     </row>
     <row r="83">
       <c r="A83" s="1"/>
@@ -2638,6 +2877,8 @@
       <c r="O83" s="1"/>
       <c r="P83" s="1"/>
       <c r="Q83" s="1"/>
+      <c r="R83" s="1"/>
+      <c r="S83" s="1"/>
     </row>
     <row r="84">
       <c r="A84" s="1"/>
@@ -2657,6 +2898,8 @@
       <c r="O84" s="1"/>
       <c r="P84" s="1"/>
       <c r="Q84" s="1"/>
+      <c r="R84" s="1"/>
+      <c r="S84" s="1"/>
     </row>
     <row r="85">
       <c r="A85" s="1"/>
@@ -2676,6 +2919,8 @@
       <c r="O85" s="1"/>
       <c r="P85" s="1"/>
       <c r="Q85" s="1"/>
+      <c r="R85" s="1"/>
+      <c r="S85" s="1"/>
     </row>
     <row r="86">
       <c r="A86" s="1"/>
@@ -2695,6 +2940,8 @@
       <c r="O86" s="1"/>
       <c r="P86" s="1"/>
       <c r="Q86" s="1"/>
+      <c r="R86" s="1"/>
+      <c r="S86" s="1"/>
     </row>
     <row r="87">
       <c r="A87" s="1"/>
@@ -2714,6 +2961,8 @@
       <c r="O87" s="1"/>
       <c r="P87" s="1"/>
       <c r="Q87" s="1"/>
+      <c r="R87" s="1"/>
+      <c r="S87" s="1"/>
     </row>
     <row r="88">
       <c r="A88" s="1"/>
@@ -2733,6 +2982,8 @@
       <c r="O88" s="1"/>
       <c r="P88" s="1"/>
       <c r="Q88" s="1"/>
+      <c r="R88" s="1"/>
+      <c r="S88" s="1"/>
     </row>
     <row r="89">
       <c r="A89" s="1"/>
@@ -2752,6 +3003,8 @@
       <c r="O89" s="1"/>
       <c r="P89" s="1"/>
       <c r="Q89" s="1"/>
+      <c r="R89" s="1"/>
+      <c r="S89" s="1"/>
     </row>
     <row r="90">
       <c r="A90" s="1"/>
@@ -2771,6 +3024,8 @@
       <c r="O90" s="1"/>
       <c r="P90" s="1"/>
       <c r="Q90" s="1"/>
+      <c r="R90" s="1"/>
+      <c r="S90" s="1"/>
     </row>
     <row r="91">
       <c r="A91" s="1"/>
@@ -2790,6 +3045,8 @@
       <c r="O91" s="1"/>
       <c r="P91" s="1"/>
       <c r="Q91" s="1"/>
+      <c r="R91" s="1"/>
+      <c r="S91" s="1"/>
     </row>
     <row r="92">
       <c r="A92" s="1"/>
@@ -2809,6 +3066,8 @@
       <c r="O92" s="1"/>
       <c r="P92" s="1"/>
       <c r="Q92" s="1"/>
+      <c r="R92" s="1"/>
+      <c r="S92" s="1"/>
     </row>
     <row r="93">
       <c r="A93" s="1"/>
@@ -2828,6 +3087,8 @@
       <c r="O93" s="1"/>
       <c r="P93" s="1"/>
       <c r="Q93" s="1"/>
+      <c r="R93" s="1"/>
+      <c r="S93" s="1"/>
     </row>
     <row r="94">
       <c r="A94" s="1"/>
@@ -2847,6 +3108,8 @@
       <c r="O94" s="1"/>
       <c r="P94" s="1"/>
       <c r="Q94" s="1"/>
+      <c r="R94" s="1"/>
+      <c r="S94" s="1"/>
     </row>
     <row r="95">
       <c r="A95" s="1"/>
@@ -2866,6 +3129,8 @@
       <c r="O95" s="1"/>
       <c r="P95" s="1"/>
       <c r="Q95" s="1"/>
+      <c r="R95" s="1"/>
+      <c r="S95" s="1"/>
     </row>
     <row r="96">
       <c r="A96" s="1"/>
@@ -2885,6 +3150,8 @@
       <c r="O96" s="1"/>
       <c r="P96" s="1"/>
       <c r="Q96" s="1"/>
+      <c r="R96" s="1"/>
+      <c r="S96" s="1"/>
     </row>
     <row r="97">
       <c r="A97" s="1"/>
@@ -2904,6 +3171,8 @@
       <c r="O97" s="1"/>
       <c r="P97" s="1"/>
       <c r="Q97" s="1"/>
+      <c r="R97" s="1"/>
+      <c r="S97" s="1"/>
     </row>
     <row r="98">
       <c r="A98" s="1"/>
@@ -2923,6 +3192,8 @@
       <c r="O98" s="1"/>
       <c r="P98" s="1"/>
       <c r="Q98" s="1"/>
+      <c r="R98" s="1"/>
+      <c r="S98" s="1"/>
     </row>
     <row r="99">
       <c r="A99" s="1"/>
@@ -2942,6 +3213,8 @@
       <c r="O99" s="1"/>
       <c r="P99" s="1"/>
       <c r="Q99" s="1"/>
+      <c r="R99" s="1"/>
+      <c r="S99" s="1"/>
     </row>
     <row r="100">
       <c r="A100" s="1"/>
@@ -2961,6 +3234,8 @@
       <c r="O100" s="1"/>
       <c r="P100" s="1"/>
       <c r="Q100" s="1"/>
+      <c r="R100" s="1"/>
+      <c r="S100" s="1"/>
     </row>
     <row r="101">
       <c r="A101" s="1"/>
@@ -2980,6 +3255,8 @@
       <c r="O101" s="1"/>
       <c r="P101" s="1"/>
       <c r="Q101" s="1"/>
+      <c r="R101" s="1"/>
+      <c r="S101" s="1"/>
     </row>
     <row r="102">
       <c r="A102" s="1"/>
@@ -2999,6 +3276,8 @@
       <c r="O102" s="1"/>
       <c r="P102" s="1"/>
       <c r="Q102" s="1"/>
+      <c r="R102" s="1"/>
+      <c r="S102" s="1"/>
     </row>
     <row r="103">
       <c r="A103" s="1"/>
@@ -3018,6 +3297,8 @@
       <c r="O103" s="1"/>
       <c r="P103" s="1"/>
       <c r="Q103" s="1"/>
+      <c r="R103" s="1"/>
+      <c r="S103" s="1"/>
     </row>
     <row r="104">
       <c r="A104" s="1"/>
@@ -3037,6 +3318,8 @@
       <c r="O104" s="1"/>
       <c r="P104" s="1"/>
       <c r="Q104" s="1"/>
+      <c r="R104" s="1"/>
+      <c r="S104" s="1"/>
     </row>
     <row r="105">
       <c r="A105" s="1"/>
@@ -3056,6 +3339,8 @@
       <c r="O105" s="1"/>
       <c r="P105" s="1"/>
       <c r="Q105" s="1"/>
+      <c r="R105" s="1"/>
+      <c r="S105" s="1"/>
     </row>
     <row r="106">
       <c r="A106" s="1"/>
@@ -3075,6 +3360,8 @@
       <c r="O106" s="1"/>
       <c r="P106" s="1"/>
       <c r="Q106" s="1"/>
+      <c r="R106" s="1"/>
+      <c r="S106" s="1"/>
     </row>
     <row r="107">
       <c r="A107" s="1"/>
@@ -3094,6 +3381,8 @@
       <c r="O107" s="1"/>
       <c r="P107" s="1"/>
       <c r="Q107" s="1"/>
+      <c r="R107" s="1"/>
+      <c r="S107" s="1"/>
     </row>
     <row r="108">
       <c r="A108" s="1"/>
@@ -3113,6 +3402,8 @@
       <c r="O108" s="1"/>
       <c r="P108" s="1"/>
       <c r="Q108" s="1"/>
+      <c r="R108" s="1"/>
+      <c r="S108" s="1"/>
     </row>
     <row r="109">
       <c r="A109" s="1"/>
@@ -3132,6 +3423,8 @@
       <c r="O109" s="1"/>
       <c r="P109" s="1"/>
       <c r="Q109" s="1"/>
+      <c r="R109" s="1"/>
+      <c r="S109" s="1"/>
     </row>
     <row r="110">
       <c r="A110" s="1"/>
@@ -3151,6 +3444,8 @@
       <c r="O110" s="1"/>
       <c r="P110" s="1"/>
       <c r="Q110" s="1"/>
+      <c r="R110" s="1"/>
+      <c r="S110" s="1"/>
     </row>
     <row r="111">
       <c r="A111" s="1"/>
@@ -3170,6 +3465,8 @@
       <c r="O111" s="1"/>
       <c r="P111" s="1"/>
       <c r="Q111" s="1"/>
+      <c r="R111" s="1"/>
+      <c r="S111" s="1"/>
     </row>
     <row r="112">
       <c r="A112" s="1"/>
@@ -3189,6 +3486,8 @@
       <c r="O112" s="1"/>
       <c r="P112" s="1"/>
       <c r="Q112" s="1"/>
+      <c r="R112" s="1"/>
+      <c r="S112" s="1"/>
     </row>
     <row r="113">
       <c r="A113" s="1"/>
@@ -3208,6 +3507,8 @@
       <c r="O113" s="1"/>
       <c r="P113" s="1"/>
       <c r="Q113" s="1"/>
+      <c r="R113" s="1"/>
+      <c r="S113" s="1"/>
     </row>
     <row r="114">
       <c r="A114" s="1"/>
@@ -3227,6 +3528,8 @@
       <c r="O114" s="1"/>
       <c r="P114" s="1"/>
       <c r="Q114" s="1"/>
+      <c r="R114" s="1"/>
+      <c r="S114" s="1"/>
     </row>
     <row r="115">
       <c r="A115" s="1"/>
@@ -3246,6 +3549,8 @@
       <c r="O115" s="1"/>
       <c r="P115" s="1"/>
       <c r="Q115" s="1"/>
+      <c r="R115" s="1"/>
+      <c r="S115" s="1"/>
     </row>
     <row r="116">
       <c r="A116" s="1"/>
@@ -3265,6 +3570,8 @@
       <c r="O116" s="1"/>
       <c r="P116" s="1"/>
       <c r="Q116" s="1"/>
+      <c r="R116" s="1"/>
+      <c r="S116" s="1"/>
     </row>
     <row r="117">
       <c r="A117" s="1"/>
@@ -3284,6 +3591,8 @@
       <c r="O117" s="1"/>
       <c r="P117" s="1"/>
       <c r="Q117" s="1"/>
+      <c r="R117" s="1"/>
+      <c r="S117" s="1"/>
     </row>
     <row r="118">
       <c r="A118" s="1"/>
@@ -3303,6 +3612,8 @@
       <c r="O118" s="1"/>
       <c r="P118" s="1"/>
       <c r="Q118" s="1"/>
+      <c r="R118" s="1"/>
+      <c r="S118" s="1"/>
     </row>
     <row r="119">
       <c r="A119" s="1"/>
@@ -3322,6 +3633,8 @@
       <c r="O119" s="1"/>
       <c r="P119" s="1"/>
       <c r="Q119" s="1"/>
+      <c r="R119" s="1"/>
+      <c r="S119" s="1"/>
     </row>
     <row r="120">
       <c r="A120" s="1"/>
@@ -3341,6 +3654,8 @@
       <c r="O120" s="1"/>
       <c r="P120" s="1"/>
       <c r="Q120" s="1"/>
+      <c r="R120" s="1"/>
+      <c r="S120" s="1"/>
     </row>
     <row r="121">
       <c r="A121" s="1"/>
@@ -3360,6 +3675,8 @@
       <c r="O121" s="1"/>
       <c r="P121" s="1"/>
       <c r="Q121" s="1"/>
+      <c r="R121" s="1"/>
+      <c r="S121" s="1"/>
     </row>
     <row r="122">
       <c r="A122" s="1"/>
@@ -3379,6 +3696,8 @@
       <c r="O122" s="1"/>
       <c r="P122" s="1"/>
       <c r="Q122" s="1"/>
+      <c r="R122" s="1"/>
+      <c r="S122" s="1"/>
     </row>
     <row r="123">
       <c r="A123" s="1"/>
@@ -3398,6 +3717,8 @@
       <c r="O123" s="1"/>
       <c r="P123" s="1"/>
       <c r="Q123" s="1"/>
+      <c r="R123" s="1"/>
+      <c r="S123" s="1"/>
     </row>
     <row r="124">
       <c r="A124" s="1"/>
@@ -3417,6 +3738,8 @@
       <c r="O124" s="1"/>
       <c r="P124" s="1"/>
       <c r="Q124" s="1"/>
+      <c r="R124" s="1"/>
+      <c r="S124" s="1"/>
     </row>
     <row r="125">
       <c r="A125" s="1"/>
@@ -3436,6 +3759,8 @@
       <c r="O125" s="1"/>
       <c r="P125" s="1"/>
       <c r="Q125" s="1"/>
+      <c r="R125" s="1"/>
+      <c r="S125" s="1"/>
     </row>
     <row r="126">
       <c r="A126" s="1"/>
@@ -3455,6 +3780,8 @@
       <c r="O126" s="1"/>
       <c r="P126" s="1"/>
       <c r="Q126" s="1"/>
+      <c r="R126" s="1"/>
+      <c r="S126" s="1"/>
     </row>
     <row r="127">
       <c r="A127" s="1"/>
@@ -3474,6 +3801,8 @@
       <c r="O127" s="1"/>
       <c r="P127" s="1"/>
       <c r="Q127" s="1"/>
+      <c r="R127" s="1"/>
+      <c r="S127" s="1"/>
     </row>
     <row r="128">
       <c r="A128" s="1"/>
@@ -3493,6 +3822,8 @@
       <c r="O128" s="1"/>
       <c r="P128" s="1"/>
       <c r="Q128" s="1"/>
+      <c r="R128" s="1"/>
+      <c r="S128" s="1"/>
     </row>
     <row r="129">
       <c r="A129" s="1"/>
@@ -3512,6 +3843,8 @@
       <c r="O129" s="1"/>
       <c r="P129" s="1"/>
       <c r="Q129" s="1"/>
+      <c r="R129" s="1"/>
+      <c r="S129" s="1"/>
     </row>
     <row r="130">
       <c r="A130" s="1"/>
@@ -3531,6 +3864,8 @@
       <c r="O130" s="1"/>
       <c r="P130" s="1"/>
       <c r="Q130" s="1"/>
+      <c r="R130" s="1"/>
+      <c r="S130" s="1"/>
     </row>
     <row r="131">
       <c r="A131" s="1"/>
@@ -3550,6 +3885,8 @@
       <c r="O131" s="1"/>
       <c r="P131" s="1"/>
       <c r="Q131" s="1"/>
+      <c r="R131" s="1"/>
+      <c r="S131" s="1"/>
     </row>
     <row r="132">
       <c r="A132" s="1"/>
@@ -3569,6 +3906,8 @@
       <c r="O132" s="1"/>
       <c r="P132" s="1"/>
       <c r="Q132" s="1"/>
+      <c r="R132" s="1"/>
+      <c r="S132" s="1"/>
     </row>
     <row r="133">
       <c r="A133" s="1"/>
@@ -3588,6 +3927,8 @@
       <c r="O133" s="1"/>
       <c r="P133" s="1"/>
       <c r="Q133" s="1"/>
+      <c r="R133" s="1"/>
+      <c r="S133" s="1"/>
     </row>
     <row r="134">
       <c r="A134" s="1"/>
@@ -3607,6 +3948,8 @@
       <c r="O134" s="1"/>
       <c r="P134" s="1"/>
       <c r="Q134" s="1"/>
+      <c r="R134" s="1"/>
+      <c r="S134" s="1"/>
     </row>
     <row r="135">
       <c r="A135" s="1"/>
@@ -3626,6 +3969,8 @@
       <c r="O135" s="1"/>
       <c r="P135" s="1"/>
       <c r="Q135" s="1"/>
+      <c r="R135" s="1"/>
+      <c r="S135" s="1"/>
     </row>
     <row r="136">
       <c r="A136" s="1"/>
@@ -3645,6 +3990,8 @@
       <c r="O136" s="1"/>
       <c r="P136" s="1"/>
       <c r="Q136" s="1"/>
+      <c r="R136" s="1"/>
+      <c r="S136" s="1"/>
     </row>
     <row r="137">
       <c r="A137" s="1"/>
@@ -3664,6 +4011,8 @@
       <c r="O137" s="1"/>
       <c r="P137" s="1"/>
       <c r="Q137" s="1"/>
+      <c r="R137" s="1"/>
+      <c r="S137" s="1"/>
     </row>
     <row r="138">
       <c r="A138" s="1"/>
@@ -3683,6 +4032,8 @@
       <c r="O138" s="1"/>
       <c r="P138" s="1"/>
       <c r="Q138" s="1"/>
+      <c r="R138" s="1"/>
+      <c r="S138" s="1"/>
     </row>
     <row r="139">
       <c r="A139" s="1"/>
@@ -3702,6 +4053,8 @@
       <c r="O139" s="1"/>
       <c r="P139" s="1"/>
       <c r="Q139" s="1"/>
+      <c r="R139" s="1"/>
+      <c r="S139" s="1"/>
     </row>
     <row r="140">
       <c r="A140" s="1"/>
@@ -3721,6 +4074,8 @@
       <c r="O140" s="1"/>
       <c r="P140" s="1"/>
       <c r="Q140" s="1"/>
+      <c r="R140" s="1"/>
+      <c r="S140" s="1"/>
     </row>
     <row r="141">
       <c r="A141" s="1"/>
@@ -3740,6 +4095,8 @@
       <c r="O141" s="1"/>
       <c r="P141" s="1"/>
       <c r="Q141" s="1"/>
+      <c r="R141" s="1"/>
+      <c r="S141" s="1"/>
     </row>
     <row r="142">
       <c r="A142" s="1"/>
@@ -3759,6 +4116,8 @@
       <c r="O142" s="1"/>
       <c r="P142" s="1"/>
       <c r="Q142" s="1"/>
+      <c r="R142" s="1"/>
+      <c r="S142" s="1"/>
     </row>
     <row r="143">
       <c r="A143" s="1"/>
@@ -3778,6 +4137,8 @@
       <c r="O143" s="1"/>
       <c r="P143" s="1"/>
       <c r="Q143" s="1"/>
+      <c r="R143" s="1"/>
+      <c r="S143" s="1"/>
     </row>
     <row r="144">
       <c r="A144" s="1"/>
@@ -3797,6 +4158,8 @@
       <c r="O144" s="1"/>
       <c r="P144" s="1"/>
       <c r="Q144" s="1"/>
+      <c r="R144" s="1"/>
+      <c r="S144" s="1"/>
     </row>
     <row r="145">
       <c r="A145" s="1"/>
@@ -3816,6 +4179,8 @@
       <c r="O145" s="1"/>
       <c r="P145" s="1"/>
       <c r="Q145" s="1"/>
+      <c r="R145" s="1"/>
+      <c r="S145" s="1"/>
     </row>
     <row r="146">
       <c r="A146" s="1"/>
@@ -3835,6 +4200,8 @@
       <c r="O146" s="1"/>
       <c r="P146" s="1"/>
       <c r="Q146" s="1"/>
+      <c r="R146" s="1"/>
+      <c r="S146" s="1"/>
     </row>
     <row r="147">
       <c r="A147" s="1"/>
@@ -3854,6 +4221,8 @@
       <c r="O147" s="1"/>
       <c r="P147" s="1"/>
       <c r="Q147" s="1"/>
+      <c r="R147" s="1"/>
+      <c r="S147" s="1"/>
     </row>
     <row r="148">
       <c r="A148" s="1"/>
@@ -3873,6 +4242,8 @@
       <c r="O148" s="1"/>
       <c r="P148" s="1"/>
       <c r="Q148" s="1"/>
+      <c r="R148" s="1"/>
+      <c r="S148" s="1"/>
     </row>
     <row r="149">
       <c r="A149" s="1"/>
@@ -3892,6 +4263,8 @@
       <c r="O149" s="1"/>
       <c r="P149" s="1"/>
       <c r="Q149" s="1"/>
+      <c r="R149" s="1"/>
+      <c r="S149" s="1"/>
     </row>
     <row r="150">
       <c r="A150" s="1"/>
@@ -3911,6 +4284,8 @@
       <c r="O150" s="1"/>
       <c r="P150" s="1"/>
       <c r="Q150" s="1"/>
+      <c r="R150" s="1"/>
+      <c r="S150" s="1"/>
     </row>
     <row r="151">
       <c r="A151" s="1"/>
@@ -3930,6 +4305,8 @@
       <c r="O151" s="1"/>
       <c r="P151" s="1"/>
       <c r="Q151" s="1"/>
+      <c r="R151" s="1"/>
+      <c r="S151" s="1"/>
     </row>
     <row r="152">
       <c r="A152" s="1"/>
@@ -3949,6 +4326,8 @@
       <c r="O152" s="1"/>
       <c r="P152" s="1"/>
       <c r="Q152" s="1"/>
+      <c r="R152" s="1"/>
+      <c r="S152" s="1"/>
     </row>
     <row r="153">
       <c r="A153" s="1"/>
@@ -3968,6 +4347,8 @@
       <c r="O153" s="1"/>
       <c r="P153" s="1"/>
       <c r="Q153" s="1"/>
+      <c r="R153" s="1"/>
+      <c r="S153" s="1"/>
     </row>
     <row r="154">
       <c r="A154" s="1"/>
@@ -3987,6 +4368,8 @@
       <c r="O154" s="1"/>
       <c r="P154" s="1"/>
       <c r="Q154" s="1"/>
+      <c r="R154" s="1"/>
+      <c r="S154" s="1"/>
     </row>
     <row r="155">
       <c r="A155" s="1"/>
@@ -4006,6 +4389,8 @@
       <c r="O155" s="1"/>
       <c r="P155" s="1"/>
       <c r="Q155" s="1"/>
+      <c r="R155" s="1"/>
+      <c r="S155" s="1"/>
     </row>
     <row r="156">
       <c r="A156" s="1"/>
@@ -4025,6 +4410,8 @@
       <c r="O156" s="1"/>
       <c r="P156" s="1"/>
       <c r="Q156" s="1"/>
+      <c r="R156" s="1"/>
+      <c r="S156" s="1"/>
     </row>
     <row r="157">
       <c r="A157" s="1"/>
@@ -4044,6 +4431,8 @@
       <c r="O157" s="1"/>
       <c r="P157" s="1"/>
       <c r="Q157" s="1"/>
+      <c r="R157" s="1"/>
+      <c r="S157" s="1"/>
     </row>
     <row r="158">
       <c r="A158" s="1"/>
@@ -4063,6 +4452,8 @@
       <c r="O158" s="1"/>
       <c r="P158" s="1"/>
       <c r="Q158" s="1"/>
+      <c r="R158" s="1"/>
+      <c r="S158" s="1"/>
     </row>
     <row r="159">
       <c r="A159" s="1"/>
@@ -4082,6 +4473,8 @@
       <c r="O159" s="1"/>
       <c r="P159" s="1"/>
       <c r="Q159" s="1"/>
+      <c r="R159" s="1"/>
+      <c r="S159" s="1"/>
     </row>
     <row r="160">
       <c r="A160" s="1"/>
@@ -4101,6 +4494,8 @@
       <c r="O160" s="1"/>
       <c r="P160" s="1"/>
       <c r="Q160" s="1"/>
+      <c r="R160" s="1"/>
+      <c r="S160" s="1"/>
     </row>
     <row r="161">
       <c r="A161" s="1"/>
@@ -4120,6 +4515,8 @@
       <c r="O161" s="1"/>
       <c r="P161" s="1"/>
       <c r="Q161" s="1"/>
+      <c r="R161" s="1"/>
+      <c r="S161" s="1"/>
     </row>
     <row r="162">
       <c r="A162" s="1"/>
@@ -4139,6 +4536,8 @@
       <c r="O162" s="1"/>
       <c r="P162" s="1"/>
       <c r="Q162" s="1"/>
+      <c r="R162" s="1"/>
+      <c r="S162" s="1"/>
     </row>
     <row r="163">
       <c r="A163" s="1"/>
@@ -4158,6 +4557,8 @@
       <c r="O163" s="1"/>
       <c r="P163" s="1"/>
       <c r="Q163" s="1"/>
+      <c r="R163" s="1"/>
+      <c r="S163" s="1"/>
     </row>
     <row r="164">
       <c r="A164" s="1"/>
@@ -4177,6 +4578,8 @@
       <c r="O164" s="1"/>
       <c r="P164" s="1"/>
       <c r="Q164" s="1"/>
+      <c r="R164" s="1"/>
+      <c r="S164" s="1"/>
     </row>
     <row r="165">
       <c r="A165" s="1"/>
@@ -4196,6 +4599,8 @@
       <c r="O165" s="1"/>
       <c r="P165" s="1"/>
       <c r="Q165" s="1"/>
+      <c r="R165" s="1"/>
+      <c r="S165" s="1"/>
     </row>
     <row r="166">
       <c r="A166" s="1"/>
@@ -4215,6 +4620,8 @@
       <c r="O166" s="1"/>
       <c r="P166" s="1"/>
       <c r="Q166" s="1"/>
+      <c r="R166" s="1"/>
+      <c r="S166" s="1"/>
     </row>
     <row r="167">
       <c r="A167" s="1"/>
@@ -4234,6 +4641,8 @@
       <c r="O167" s="1"/>
       <c r="P167" s="1"/>
       <c r="Q167" s="1"/>
+      <c r="R167" s="1"/>
+      <c r="S167" s="1"/>
     </row>
     <row r="168">
       <c r="A168" s="1"/>
@@ -4253,6 +4662,8 @@
       <c r="O168" s="1"/>
       <c r="P168" s="1"/>
       <c r="Q168" s="1"/>
+      <c r="R168" s="1"/>
+      <c r="S168" s="1"/>
     </row>
     <row r="169">
       <c r="A169" s="1"/>
@@ -4272,6 +4683,8 @@
       <c r="O169" s="1"/>
       <c r="P169" s="1"/>
       <c r="Q169" s="1"/>
+      <c r="R169" s="1"/>
+      <c r="S169" s="1"/>
     </row>
     <row r="170">
       <c r="A170" s="1"/>
@@ -4291,6 +4704,8 @@
       <c r="O170" s="1"/>
       <c r="P170" s="1"/>
       <c r="Q170" s="1"/>
+      <c r="R170" s="1"/>
+      <c r="S170" s="1"/>
     </row>
     <row r="171">
       <c r="A171" s="1"/>
@@ -4310,6 +4725,8 @@
       <c r="O171" s="1"/>
       <c r="P171" s="1"/>
       <c r="Q171" s="1"/>
+      <c r="R171" s="1"/>
+      <c r="S171" s="1"/>
     </row>
     <row r="172">
       <c r="A172" s="1"/>
@@ -4329,6 +4746,8 @@
       <c r="O172" s="1"/>
       <c r="P172" s="1"/>
       <c r="Q172" s="1"/>
+      <c r="R172" s="1"/>
+      <c r="S172" s="1"/>
     </row>
     <row r="173">
       <c r="A173" s="1"/>
@@ -4348,6 +4767,8 @@
       <c r="O173" s="1"/>
       <c r="P173" s="1"/>
       <c r="Q173" s="1"/>
+      <c r="R173" s="1"/>
+      <c r="S173" s="1"/>
     </row>
     <row r="174">
       <c r="A174" s="1"/>
@@ -4367,6 +4788,8 @@
       <c r="O174" s="1"/>
       <c r="P174" s="1"/>
       <c r="Q174" s="1"/>
+      <c r="R174" s="1"/>
+      <c r="S174" s="1"/>
     </row>
     <row r="175">
       <c r="A175" s="1"/>
@@ -4386,6 +4809,8 @@
       <c r="O175" s="1"/>
       <c r="P175" s="1"/>
       <c r="Q175" s="1"/>
+      <c r="R175" s="1"/>
+      <c r="S175" s="1"/>
     </row>
     <row r="176">
       <c r="A176" s="1"/>
@@ -4405,6 +4830,8 @@
       <c r="O176" s="1"/>
       <c r="P176" s="1"/>
       <c r="Q176" s="1"/>
+      <c r="R176" s="1"/>
+      <c r="S176" s="1"/>
     </row>
     <row r="177">
       <c r="A177" s="1"/>
@@ -4424,6 +4851,8 @@
       <c r="O177" s="1"/>
       <c r="P177" s="1"/>
       <c r="Q177" s="1"/>
+      <c r="R177" s="1"/>
+      <c r="S177" s="1"/>
     </row>
     <row r="178">
       <c r="A178" s="1"/>
@@ -4443,6 +4872,8 @@
       <c r="O178" s="1"/>
       <c r="P178" s="1"/>
       <c r="Q178" s="1"/>
+      <c r="R178" s="1"/>
+      <c r="S178" s="1"/>
     </row>
     <row r="179">
       <c r="A179" s="1"/>
@@ -4462,6 +4893,8 @@
       <c r="O179" s="1"/>
       <c r="P179" s="1"/>
       <c r="Q179" s="1"/>
+      <c r="R179" s="1"/>
+      <c r="S179" s="1"/>
     </row>
     <row r="180">
       <c r="A180" s="1"/>
@@ -4481,6 +4914,8 @@
       <c r="O180" s="1"/>
       <c r="P180" s="1"/>
       <c r="Q180" s="1"/>
+      <c r="R180" s="1"/>
+      <c r="S180" s="1"/>
     </row>
     <row r="181">
       <c r="A181" s="1"/>
@@ -4500,6 +4935,8 @@
       <c r="O181" s="1"/>
       <c r="P181" s="1"/>
       <c r="Q181" s="1"/>
+      <c r="R181" s="1"/>
+      <c r="S181" s="1"/>
     </row>
     <row r="182">
       <c r="A182" s="1"/>
@@ -4519,6 +4956,8 @@
       <c r="O182" s="1"/>
       <c r="P182" s="1"/>
       <c r="Q182" s="1"/>
+      <c r="R182" s="1"/>
+      <c r="S182" s="1"/>
     </row>
     <row r="183">
       <c r="A183" s="1"/>
@@ -4538,6 +4977,8 @@
       <c r="O183" s="1"/>
       <c r="P183" s="1"/>
       <c r="Q183" s="1"/>
+      <c r="R183" s="1"/>
+      <c r="S183" s="1"/>
     </row>
     <row r="184">
       <c r="A184" s="1"/>
@@ -4557,6 +4998,8 @@
       <c r="O184" s="1"/>
       <c r="P184" s="1"/>
       <c r="Q184" s="1"/>
+      <c r="R184" s="1"/>
+      <c r="S184" s="1"/>
     </row>
     <row r="185">
       <c r="A185" s="1"/>
@@ -4576,6 +5019,8 @@
       <c r="O185" s="1"/>
       <c r="P185" s="1"/>
       <c r="Q185" s="1"/>
+      <c r="R185" s="1"/>
+      <c r="S185" s="1"/>
     </row>
     <row r="186">
       <c r="A186" s="1"/>
@@ -4595,6 +5040,8 @@
       <c r="O186" s="1"/>
       <c r="P186" s="1"/>
       <c r="Q186" s="1"/>
+      <c r="R186" s="1"/>
+      <c r="S186" s="1"/>
     </row>
     <row r="187">
       <c r="A187" s="1"/>
@@ -4614,6 +5061,8 @@
       <c r="O187" s="1"/>
       <c r="P187" s="1"/>
       <c r="Q187" s="1"/>
+      <c r="R187" s="1"/>
+      <c r="S187" s="1"/>
     </row>
     <row r="188">
       <c r="A188" s="1"/>
@@ -4633,6 +5082,8 @@
       <c r="O188" s="1"/>
       <c r="P188" s="1"/>
       <c r="Q188" s="1"/>
+      <c r="R188" s="1"/>
+      <c r="S188" s="1"/>
     </row>
     <row r="189">
       <c r="A189" s="1"/>
@@ -4652,6 +5103,8 @@
       <c r="O189" s="1"/>
       <c r="P189" s="1"/>
       <c r="Q189" s="1"/>
+      <c r="R189" s="1"/>
+      <c r="S189" s="1"/>
     </row>
     <row r="190">
       <c r="A190" s="1"/>
@@ -4671,6 +5124,8 @@
       <c r="O190" s="1"/>
       <c r="P190" s="1"/>
       <c r="Q190" s="1"/>
+      <c r="R190" s="1"/>
+      <c r="S190" s="1"/>
     </row>
     <row r="191">
       <c r="A191" s="1"/>
@@ -4690,6 +5145,8 @@
       <c r="O191" s="1"/>
       <c r="P191" s="1"/>
       <c r="Q191" s="1"/>
+      <c r="R191" s="1"/>
+      <c r="S191" s="1"/>
     </row>
     <row r="192">
       <c r="A192" s="1"/>
@@ -4709,6 +5166,8 @@
       <c r="O192" s="1"/>
       <c r="P192" s="1"/>
       <c r="Q192" s="1"/>
+      <c r="R192" s="1"/>
+      <c r="S192" s="1"/>
     </row>
     <row r="193">
       <c r="A193" s="1"/>
@@ -4728,6 +5187,8 @@
       <c r="O193" s="1"/>
       <c r="P193" s="1"/>
       <c r="Q193" s="1"/>
+      <c r="R193" s="1"/>
+      <c r="S193" s="1"/>
     </row>
     <row r="194">
       <c r="A194" s="1"/>
@@ -4747,6 +5208,8 @@
       <c r="O194" s="1"/>
       <c r="P194" s="1"/>
       <c r="Q194" s="1"/>
+      <c r="R194" s="1"/>
+      <c r="S194" s="1"/>
     </row>
     <row r="195">
       <c r="A195" s="1"/>
@@ -4766,6 +5229,8 @@
       <c r="O195" s="1"/>
       <c r="P195" s="1"/>
       <c r="Q195" s="1"/>
+      <c r="R195" s="1"/>
+      <c r="S195" s="1"/>
     </row>
     <row r="196">
       <c r="A196" s="1"/>
@@ -4785,6 +5250,8 @@
       <c r="O196" s="1"/>
       <c r="P196" s="1"/>
       <c r="Q196" s="1"/>
+      <c r="R196" s="1"/>
+      <c r="S196" s="1"/>
     </row>
     <row r="197">
       <c r="A197" s="1"/>
@@ -4804,6 +5271,8 @@
       <c r="O197" s="1"/>
       <c r="P197" s="1"/>
       <c r="Q197" s="1"/>
+      <c r="R197" s="1"/>
+      <c r="S197" s="1"/>
     </row>
     <row r="198">
       <c r="A198" s="1"/>
@@ -4823,6 +5292,8 @@
       <c r="O198" s="1"/>
       <c r="P198" s="1"/>
       <c r="Q198" s="1"/>
+      <c r="R198" s="1"/>
+      <c r="S198" s="1"/>
     </row>
     <row r="199">
       <c r="A199" s="1"/>
@@ -4842,6 +5313,8 @@
       <c r="O199" s="1"/>
       <c r="P199" s="1"/>
       <c r="Q199" s="1"/>
+      <c r="R199" s="1"/>
+      <c r="S199" s="1"/>
     </row>
     <row r="200">
       <c r="A200" s="1"/>
@@ -4861,6 +5334,8 @@
       <c r="O200" s="1"/>
       <c r="P200" s="1"/>
       <c r="Q200" s="1"/>
+      <c r="R200" s="1"/>
+      <c r="S200" s="1"/>
     </row>
     <row r="201">
       <c r="A201" s="1"/>
@@ -4880,6 +5355,8 @@
       <c r="O201" s="1"/>
       <c r="P201" s="1"/>
       <c r="Q201" s="1"/>
+      <c r="R201" s="1"/>
+      <c r="S201" s="1"/>
     </row>
     <row r="202">
       <c r="A202" s="1"/>
@@ -4899,6 +5376,8 @@
       <c r="O202" s="1"/>
       <c r="P202" s="1"/>
       <c r="Q202" s="1"/>
+      <c r="R202" s="1"/>
+      <c r="S202" s="1"/>
     </row>
     <row r="203">
       <c r="A203" s="1"/>
@@ -4918,6 +5397,8 @@
       <c r="O203" s="1"/>
       <c r="P203" s="1"/>
       <c r="Q203" s="1"/>
+      <c r="R203" s="1"/>
+      <c r="S203" s="1"/>
     </row>
     <row r="204">
       <c r="A204" s="1"/>
@@ -4937,6 +5418,8 @@
       <c r="O204" s="1"/>
       <c r="P204" s="1"/>
       <c r="Q204" s="1"/>
+      <c r="R204" s="1"/>
+      <c r="S204" s="1"/>
     </row>
     <row r="205">
       <c r="A205" s="1"/>
@@ -4956,6 +5439,8 @@
       <c r="O205" s="1"/>
       <c r="P205" s="1"/>
       <c r="Q205" s="1"/>
+      <c r="R205" s="1"/>
+      <c r="S205" s="1"/>
     </row>
     <row r="206">
       <c r="A206" s="1"/>
@@ -4975,6 +5460,8 @@
       <c r="O206" s="1"/>
       <c r="P206" s="1"/>
       <c r="Q206" s="1"/>
+      <c r="R206" s="1"/>
+      <c r="S206" s="1"/>
     </row>
     <row r="207">
       <c r="A207" s="1"/>
@@ -4994,6 +5481,8 @@
       <c r="O207" s="1"/>
       <c r="P207" s="1"/>
       <c r="Q207" s="1"/>
+      <c r="R207" s="1"/>
+      <c r="S207" s="1"/>
     </row>
     <row r="208">
       <c r="A208" s="1"/>
@@ -5013,6 +5502,8 @@
       <c r="O208" s="1"/>
       <c r="P208" s="1"/>
       <c r="Q208" s="1"/>
+      <c r="R208" s="1"/>
+      <c r="S208" s="1"/>
     </row>
     <row r="209">
       <c r="A209" s="1"/>
@@ -5032,6 +5523,8 @@
       <c r="O209" s="1"/>
       <c r="P209" s="1"/>
       <c r="Q209" s="1"/>
+      <c r="R209" s="1"/>
+      <c r="S209" s="1"/>
     </row>
     <row r="210">
       <c r="A210" s="1"/>
@@ -5051,6 +5544,8 @@
       <c r="O210" s="1"/>
       <c r="P210" s="1"/>
       <c r="Q210" s="1"/>
+      <c r="R210" s="1"/>
+      <c r="S210" s="1"/>
     </row>
     <row r="211">
       <c r="A211" s="1"/>
@@ -5070,6 +5565,8 @@
       <c r="O211" s="1"/>
       <c r="P211" s="1"/>
       <c r="Q211" s="1"/>
+      <c r="R211" s="1"/>
+      <c r="S211" s="1"/>
     </row>
     <row r="212">
       <c r="A212" s="1"/>
@@ -5089,6 +5586,8 @@
       <c r="O212" s="1"/>
       <c r="P212" s="1"/>
       <c r="Q212" s="1"/>
+      <c r="R212" s="1"/>
+      <c r="S212" s="1"/>
     </row>
     <row r="213">
       <c r="A213" s="1"/>
@@ -5108,6 +5607,8 @@
       <c r="O213" s="1"/>
       <c r="P213" s="1"/>
       <c r="Q213" s="1"/>
+      <c r="R213" s="1"/>
+      <c r="S213" s="1"/>
     </row>
     <row r="214">
       <c r="A214" s="1"/>
@@ -5127,6 +5628,8 @@
       <c r="O214" s="1"/>
       <c r="P214" s="1"/>
       <c r="Q214" s="1"/>
+      <c r="R214" s="1"/>
+      <c r="S214" s="1"/>
     </row>
     <row r="215">
       <c r="A215" s="1"/>
@@ -5146,6 +5649,8 @@
       <c r="O215" s="1"/>
       <c r="P215" s="1"/>
       <c r="Q215" s="1"/>
+      <c r="R215" s="1"/>
+      <c r="S215" s="1"/>
     </row>
     <row r="216">
       <c r="A216" s="1"/>
@@ -5165,9 +5670,11 @@
       <c r="O216" s="1"/>
       <c r="P216" s="1"/>
       <c r="Q216" s="1"/>
+      <c r="R216" s="1"/>
+      <c r="S216" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:S16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
data: review DiA 2008 organizations
15 rows checked against dia_2008_organizations.html.
- 2 edited: edits to `endorser_name` and `note` to appropriately seperate organization names from descriptive notes.

Review status set to complete in data_sources.md.
</commit_message>
<xml_diff>
--- a/data/raw/Democracy in Action/review/dia_2008_organizations_review.xlsx
+++ b/data/raw/Democracy in Action/review/dia_2008_organizations_review.xlsx
@@ -1,358 +1,368 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katherineparslow/Documents/repos/presidential-endorsements/data/raw/Democracy in Action/review/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D63F34-9AAA-BF46-A8C9-87E8AB4D4F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="review" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="review" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'review'!$A$1:$S$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">review!$A$1:$S$16</definedName>
   </definedNames>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
-  <si>
-    <t xml:space="preserve">row_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">review_action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">review_note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contest_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">party</t>
-  </si>
-  <si>
-    <t xml:space="preserve">endorsee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">endorser_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">endorser_description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">endorser_party_note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">district</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date_raw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">switch_direction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">switch_candidate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">evidence_url</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parsed_ok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">raw_text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">2008D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clinton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">American Nurses Association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Organization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan. 25, 2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/ana012508pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">American Nurses Association (Jan. 25, 2008)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Women's Campaign Forum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 18, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/wcf051807pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Women's Campaign Forum (May 18, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Women's Political Caucus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">April 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Women's Political Caucus (April 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Organization for Women PAC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">March 28, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/nowpac032807pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Organization for Women PAC (March 28, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMILY'S List</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan. 20, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/emilys012007pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMILY'S List (Jan. 20, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edwards</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friends of Earth Action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct. 14, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/foea101407pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friends of Earth Action (Oct. 14, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NARAL Pro-Choice America</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 14, 2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/interestg08/naral051408pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NARAL Pro-Choice America (May 14, 2008)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">American Hunters and Shooters Association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">April 16, 2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/ahsa041608pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">American Hunters and Shooters Association (April 16, 2008)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">American Small Business League</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feb. 26, 2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/asbl022608pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">American Small Business League (Feb. 26, 2008)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MoveOn.org Political Action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feb. 1, 2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/moveon020108pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MoveOn.org Political Action (Feb. 1, 2008)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armenian National Committee of America</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan. 30, 2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/anca013008pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armenian National Committee of America (Jan. 30, 2008)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2008R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giuliani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U.S. Airport and Seaport Police, a member of the International Association of Airport and Seaport Police</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sept. 7, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAASP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/giuliani/giuliani090707pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U.S. Airport and Seaport Police, a member of the International Association of Airport and Seaport Police (IAASP) (Sept. 7, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Huckabee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home School Legal Defense Association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">June 20, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/hslda062007.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home School Legal Defense Association (June 20, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">McCain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Republicans for Environmental Protection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/rep101407pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Republicans for Environmental Protection (REP) (Oct. 14, 2007)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F.Thompson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Right to Life</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov. 13, 2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://p2008.org/cands08/endorse/nrtl111307pr.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Right to Life (Nov. 13, 2007)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="111">
+  <si>
+    <t>row_id</t>
+  </si>
+  <si>
+    <t>review_action</t>
+  </si>
+  <si>
+    <t>review_note</t>
+  </si>
+  <si>
+    <t>contest_id</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>party</t>
+  </si>
+  <si>
+    <t>endorsee</t>
+  </si>
+  <si>
+    <t>endorser_name</t>
+  </si>
+  <si>
+    <t>endorser_description</t>
+  </si>
+  <si>
+    <t>endorser_party_note</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>district</t>
+  </si>
+  <si>
+    <t>date_raw</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>switch_direction</t>
+  </si>
+  <si>
+    <t>switch_candidate</t>
+  </si>
+  <si>
+    <t>evidence_url</t>
+  </si>
+  <si>
+    <t>parsed_ok</t>
+  </si>
+  <si>
+    <t>raw_text</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2008D</t>
+  </si>
+  <si>
+    <t>2008</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Clinton</t>
+  </si>
+  <si>
+    <t>American Nurses Association</t>
+  </si>
+  <si>
+    <t>National Organization</t>
+  </si>
+  <si>
+    <t>Jan. 25, 2008</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/ana012508pr.html</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>American Nurses Association (Jan. 25, 2008)</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Women's Campaign Forum</t>
+  </si>
+  <si>
+    <t>May 18, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/wcf051807pr.html</t>
+  </si>
+  <si>
+    <t>Women's Campaign Forum (May 18, 2007)</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>National Women's Political Caucus</t>
+  </si>
+  <si>
+    <t>April 2007</t>
+  </si>
+  <si>
+    <t>National Women's Political Caucus (April 2007)</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>National Organization for Women PAC</t>
+  </si>
+  <si>
+    <t>March 28, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/nowpac032807pr.html</t>
+  </si>
+  <si>
+    <t>National Organization for Women PAC (March 28, 2007)</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>EMILY'S List</t>
+  </si>
+  <si>
+    <t>Jan. 20, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/emilys012007pr.html</t>
+  </si>
+  <si>
+    <t>EMILY'S List (Jan. 20, 2007)</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Edwards</t>
+  </si>
+  <si>
+    <t>Friends of Earth Action</t>
+  </si>
+  <si>
+    <t>Oct. 14, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/foea101407pr.html</t>
+  </si>
+  <si>
+    <t>Friends of Earth Action (Oct. 14, 2007)</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Obama</t>
+  </si>
+  <si>
+    <t>NARAL Pro-Choice America</t>
+  </si>
+  <si>
+    <t>May 14, 2008</t>
+  </si>
+  <si>
+    <t>http://p2008.org/interestg08/naral051408pr.html</t>
+  </si>
+  <si>
+    <t>NARAL Pro-Choice America (May 14, 2008)</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>American Hunters and Shooters Association</t>
+  </si>
+  <si>
+    <t>April 16, 2008</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/ahsa041608pr.html</t>
+  </si>
+  <si>
+    <t>American Hunters and Shooters Association (April 16, 2008)</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>American Small Business League</t>
+  </si>
+  <si>
+    <t>Feb. 26, 2008</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/asbl022608pr.html</t>
+  </si>
+  <si>
+    <t>American Small Business League (Feb. 26, 2008)</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>MoveOn.org Political Action</t>
+  </si>
+  <si>
+    <t>Feb. 1, 2008</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/moveon020108pr.html</t>
+  </si>
+  <si>
+    <t>MoveOn.org Political Action (Feb. 1, 2008)</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Armenian National Committee of America</t>
+  </si>
+  <si>
+    <t>Jan. 30, 2008</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/anca013008pr.html</t>
+  </si>
+  <si>
+    <t>Armenian National Committee of America (Jan. 30, 2008)</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>2008R</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Giuliani</t>
+  </si>
+  <si>
+    <t>Sept. 7, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/giuliani/giuliani090707pr.html</t>
+  </si>
+  <si>
+    <t>U.S. Airport and Seaport Police, a member of the International Association of Airport and Seaport Police (IAASP) (Sept. 7, 2007)</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Huckabee</t>
+  </si>
+  <si>
+    <t>Home School Legal Defense Association</t>
+  </si>
+  <si>
+    <t>June 20, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/hslda062007.html</t>
+  </si>
+  <si>
+    <t>Home School Legal Defense Association (June 20, 2007)</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>McCain</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/rep101407pr.html</t>
+  </si>
+  <si>
+    <t>Republicans for Environmental Protection (REP) (Oct. 14, 2007)</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>F.Thompson</t>
+  </si>
+  <si>
+    <t>National Right to Life</t>
+  </si>
+  <si>
+    <t>Nov. 13, 2007</t>
+  </si>
+  <si>
+    <t>http://p2008.org/cands08/endorse/nrtl111307pr.html</t>
+  </si>
+  <si>
+    <t>National Right to Life (Nov. 13, 2007)</t>
+  </si>
+  <si>
+    <t>a member of the International Association of Airport and Seaport Police (IAASP)</t>
+  </si>
+  <si>
+    <t>U.S. Airport and Seaport Police</t>
+  </si>
+  <si>
+    <t>edited</t>
+  </si>
+  <si>
+    <t>Republicans for Environmental Protection (REP)</t>
+  </si>
+  <si>
+    <t>moved "(REP)" from `note` to `endorser_description`.</t>
+  </si>
+  <si>
+    <t>moved "a member of the International Associaition of Airport and Seaport Police" from `endorser_name` to `note`.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="@"/>
-  </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -364,12 +374,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -394,13 +406,22 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -682,32 +703,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:S216"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="8.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="8.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="12.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="40.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="23.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="21.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="8.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="10.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="16.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="18.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="18.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="40.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="11.71" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="80.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="40.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="6" width="8.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="40.6640625" customWidth="1"/>
+    <col min="9" max="9" width="23.6640625" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" customWidth="1"/>
+    <col min="11" max="11" width="8.6640625" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="14" max="14" width="8.6640625" customWidth="1"/>
+    <col min="15" max="16" width="18.6640625" customWidth="1"/>
+    <col min="17" max="17" width="40.6640625" customWidth="1"/>
+    <col min="18" max="18" width="11.6640625" customWidth="1"/>
+    <col min="19" max="19" width="80.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -766,7 +785,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -813,7 +832,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
@@ -860,7 +879,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>36</v>
       </c>
@@ -905,7 +924,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>40</v>
       </c>
@@ -952,7 +971,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
@@ -999,7 +1018,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>50</v>
       </c>
@@ -1046,7 +1065,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>56</v>
       </c>
@@ -1093,7 +1112,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>62</v>
       </c>
@@ -1140,7 +1159,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>67</v>
       </c>
@@ -1187,7 +1206,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>72</v>
       </c>
@@ -1234,7 +1253,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>77</v>
       </c>
@@ -1281,15 +1300,15 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>82</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>83</v>
@@ -1304,7 +1323,7 @@
         <v>85</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>26</v>
@@ -1313,26 +1332,26 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="R13" s="1" t="s">
         <v>29</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>20</v>
@@ -1350,10 +1369,10 @@
         <v>84</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>26</v>
@@ -1362,30 +1381,30 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="R14" s="1" t="s">
         <v>29</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>83</v>
@@ -1397,10 +1416,10 @@
         <v>84</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>26</v>
@@ -1411,24 +1430,22 @@
       <c r="M15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N15" s="1" t="s">
-        <v>100</v>
-      </c>
+      <c r="N15" s="1"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="R15" s="1" t="s">
         <v>29</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>20</v>
@@ -1446,10 +1463,10 @@
         <v>84</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>26</v>
@@ -1458,22 +1475,22 @@
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
       <c r="Q16" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="R16" s="1" t="s">
         <v>29</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1494,7 +1511,7 @@
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1515,7 +1532,7 @@
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1536,7 +1553,7 @@
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1557,7 +1574,7 @@
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1578,7 +1595,7 @@
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1599,7 +1616,7 @@
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1620,7 +1637,7 @@
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1641,7 +1658,7 @@
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1662,7 +1679,7 @@
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1683,7 +1700,7 @@
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1704,7 +1721,7 @@
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1725,7 +1742,7 @@
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1746,7 +1763,7 @@
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1767,7 +1784,7 @@
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1788,7 +1805,7 @@
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1809,7 +1826,7 @@
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1830,7 +1847,7 @@
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1851,7 +1868,7 @@
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1872,7 +1889,7 @@
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1893,7 +1910,7 @@
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1914,7 +1931,7 @@
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1935,7 +1952,7 @@
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1956,7 +1973,7 @@
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1977,7 +1994,7 @@
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1998,7 +2015,7 @@
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2019,7 +2036,7 @@
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2040,7 +2057,7 @@
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2061,7 +2078,7 @@
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2082,7 +2099,7 @@
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2103,7 +2120,7 @@
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
     </row>
-    <row r="47">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -2124,7 +2141,7 @@
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -2145,7 +2162,7 @@
       <c r="R48" s="1"/>
       <c r="S48" s="1"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -2166,7 +2183,7 @@
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -2187,7 +2204,7 @@
       <c r="R50" s="1"/>
       <c r="S50" s="1"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -2208,7 +2225,7 @@
       <c r="R51" s="1"/>
       <c r="S51" s="1"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -2229,7 +2246,7 @@
       <c r="R52" s="1"/>
       <c r="S52" s="1"/>
     </row>
-    <row r="53">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -2250,7 +2267,7 @@
       <c r="R53" s="1"/>
       <c r="S53" s="1"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -2271,7 +2288,7 @@
       <c r="R54" s="1"/>
       <c r="S54" s="1"/>
     </row>
-    <row r="55">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -2292,7 +2309,7 @@
       <c r="R55" s="1"/>
       <c r="S55" s="1"/>
     </row>
-    <row r="56">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -2313,7 +2330,7 @@
       <c r="R56" s="1"/>
       <c r="S56" s="1"/>
     </row>
-    <row r="57">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -2334,7 +2351,7 @@
       <c r="R57" s="1"/>
       <c r="S57" s="1"/>
     </row>
-    <row r="58">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -2355,7 +2372,7 @@
       <c r="R58" s="1"/>
       <c r="S58" s="1"/>
     </row>
-    <row r="59">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -2376,7 +2393,7 @@
       <c r="R59" s="1"/>
       <c r="S59" s="1"/>
     </row>
-    <row r="60">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -2397,7 +2414,7 @@
       <c r="R60" s="1"/>
       <c r="S60" s="1"/>
     </row>
-    <row r="61">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2418,7 +2435,7 @@
       <c r="R61" s="1"/>
       <c r="S61" s="1"/>
     </row>
-    <row r="62">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -2439,7 +2456,7 @@
       <c r="R62" s="1"/>
       <c r="S62" s="1"/>
     </row>
-    <row r="63">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -2460,7 +2477,7 @@
       <c r="R63" s="1"/>
       <c r="S63" s="1"/>
     </row>
-    <row r="64">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -2481,7 +2498,7 @@
       <c r="R64" s="1"/>
       <c r="S64" s="1"/>
     </row>
-    <row r="65">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -2502,7 +2519,7 @@
       <c r="R65" s="1"/>
       <c r="S65" s="1"/>
     </row>
-    <row r="66">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -2523,7 +2540,7 @@
       <c r="R66" s="1"/>
       <c r="S66" s="1"/>
     </row>
-    <row r="67">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -2544,7 +2561,7 @@
       <c r="R67" s="1"/>
       <c r="S67" s="1"/>
     </row>
-    <row r="68">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -2565,7 +2582,7 @@
       <c r="R68" s="1"/>
       <c r="S68" s="1"/>
     </row>
-    <row r="69">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -2586,7 +2603,7 @@
       <c r="R69" s="1"/>
       <c r="S69" s="1"/>
     </row>
-    <row r="70">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -2607,7 +2624,7 @@
       <c r="R70" s="1"/>
       <c r="S70" s="1"/>
     </row>
-    <row r="71">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -2628,7 +2645,7 @@
       <c r="R71" s="1"/>
       <c r="S71" s="1"/>
     </row>
-    <row r="72">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -2649,7 +2666,7 @@
       <c r="R72" s="1"/>
       <c r="S72" s="1"/>
     </row>
-    <row r="73">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -2670,7 +2687,7 @@
       <c r="R73" s="1"/>
       <c r="S73" s="1"/>
     </row>
-    <row r="74">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -2691,7 +2708,7 @@
       <c r="R74" s="1"/>
       <c r="S74" s="1"/>
     </row>
-    <row r="75">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -2712,7 +2729,7 @@
       <c r="R75" s="1"/>
       <c r="S75" s="1"/>
     </row>
-    <row r="76">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -2733,7 +2750,7 @@
       <c r="R76" s="1"/>
       <c r="S76" s="1"/>
     </row>
-    <row r="77">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -2754,7 +2771,7 @@
       <c r="R77" s="1"/>
       <c r="S77" s="1"/>
     </row>
-    <row r="78">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -2775,7 +2792,7 @@
       <c r="R78" s="1"/>
       <c r="S78" s="1"/>
     </row>
-    <row r="79">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -2796,7 +2813,7 @@
       <c r="R79" s="1"/>
       <c r="S79" s="1"/>
     </row>
-    <row r="80">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -2817,7 +2834,7 @@
       <c r="R80" s="1"/>
       <c r="S80" s="1"/>
     </row>
-    <row r="81">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -2838,7 +2855,7 @@
       <c r="R81" s="1"/>
       <c r="S81" s="1"/>
     </row>
-    <row r="82">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -2859,7 +2876,7 @@
       <c r="R82" s="1"/>
       <c r="S82" s="1"/>
     </row>
-    <row r="83">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -2880,7 +2897,7 @@
       <c r="R83" s="1"/>
       <c r="S83" s="1"/>
     </row>
-    <row r="84">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -2901,7 +2918,7 @@
       <c r="R84" s="1"/>
       <c r="S84" s="1"/>
     </row>
-    <row r="85">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -2922,7 +2939,7 @@
       <c r="R85" s="1"/>
       <c r="S85" s="1"/>
     </row>
-    <row r="86">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -2943,7 +2960,7 @@
       <c r="R86" s="1"/>
       <c r="S86" s="1"/>
     </row>
-    <row r="87">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -2964,7 +2981,7 @@
       <c r="R87" s="1"/>
       <c r="S87" s="1"/>
     </row>
-    <row r="88">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -2985,7 +3002,7 @@
       <c r="R88" s="1"/>
       <c r="S88" s="1"/>
     </row>
-    <row r="89">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -3006,7 +3023,7 @@
       <c r="R89" s="1"/>
       <c r="S89" s="1"/>
     </row>
-    <row r="90">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -3027,7 +3044,7 @@
       <c r="R90" s="1"/>
       <c r="S90" s="1"/>
     </row>
-    <row r="91">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -3048,7 +3065,7 @@
       <c r="R91" s="1"/>
       <c r="S91" s="1"/>
     </row>
-    <row r="92">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -3069,7 +3086,7 @@
       <c r="R92" s="1"/>
       <c r="S92" s="1"/>
     </row>
-    <row r="93">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -3090,7 +3107,7 @@
       <c r="R93" s="1"/>
       <c r="S93" s="1"/>
     </row>
-    <row r="94">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -3111,7 +3128,7 @@
       <c r="R94" s="1"/>
       <c r="S94" s="1"/>
     </row>
-    <row r="95">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -3132,7 +3149,7 @@
       <c r="R95" s="1"/>
       <c r="S95" s="1"/>
     </row>
-    <row r="96">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -3153,7 +3170,7 @@
       <c r="R96" s="1"/>
       <c r="S96" s="1"/>
     </row>
-    <row r="97">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -3174,7 +3191,7 @@
       <c r="R97" s="1"/>
       <c r="S97" s="1"/>
     </row>
-    <row r="98">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -3195,7 +3212,7 @@
       <c r="R98" s="1"/>
       <c r="S98" s="1"/>
     </row>
-    <row r="99">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -3216,7 +3233,7 @@
       <c r="R99" s="1"/>
       <c r="S99" s="1"/>
     </row>
-    <row r="100">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -3237,7 +3254,7 @@
       <c r="R100" s="1"/>
       <c r="S100" s="1"/>
     </row>
-    <row r="101">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -3258,7 +3275,7 @@
       <c r="R101" s="1"/>
       <c r="S101" s="1"/>
     </row>
-    <row r="102">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -3279,7 +3296,7 @@
       <c r="R102" s="1"/>
       <c r="S102" s="1"/>
     </row>
-    <row r="103">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -3300,7 +3317,7 @@
       <c r="R103" s="1"/>
       <c r="S103" s="1"/>
     </row>
-    <row r="104">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -3321,7 +3338,7 @@
       <c r="R104" s="1"/>
       <c r="S104" s="1"/>
     </row>
-    <row r="105">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -3342,7 +3359,7 @@
       <c r="R105" s="1"/>
       <c r="S105" s="1"/>
     </row>
-    <row r="106">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -3363,7 +3380,7 @@
       <c r="R106" s="1"/>
       <c r="S106" s="1"/>
     </row>
-    <row r="107">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -3384,7 +3401,7 @@
       <c r="R107" s="1"/>
       <c r="S107" s="1"/>
     </row>
-    <row r="108">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -3405,7 +3422,7 @@
       <c r="R108" s="1"/>
       <c r="S108" s="1"/>
     </row>
-    <row r="109">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -3426,7 +3443,7 @@
       <c r="R109" s="1"/>
       <c r="S109" s="1"/>
     </row>
-    <row r="110">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -3447,7 +3464,7 @@
       <c r="R110" s="1"/>
       <c r="S110" s="1"/>
     </row>
-    <row r="111">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -3468,7 +3485,7 @@
       <c r="R111" s="1"/>
       <c r="S111" s="1"/>
     </row>
-    <row r="112">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -3489,7 +3506,7 @@
       <c r="R112" s="1"/>
       <c r="S112" s="1"/>
     </row>
-    <row r="113">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -3510,7 +3527,7 @@
       <c r="R113" s="1"/>
       <c r="S113" s="1"/>
     </row>
-    <row r="114">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -3531,7 +3548,7 @@
       <c r="R114" s="1"/>
       <c r="S114" s="1"/>
     </row>
-    <row r="115">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -3552,7 +3569,7 @@
       <c r="R115" s="1"/>
       <c r="S115" s="1"/>
     </row>
-    <row r="116">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -3573,7 +3590,7 @@
       <c r="R116" s="1"/>
       <c r="S116" s="1"/>
     </row>
-    <row r="117">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -3594,7 +3611,7 @@
       <c r="R117" s="1"/>
       <c r="S117" s="1"/>
     </row>
-    <row r="118">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -3615,7 +3632,7 @@
       <c r="R118" s="1"/>
       <c r="S118" s="1"/>
     </row>
-    <row r="119">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -3636,7 +3653,7 @@
       <c r="R119" s="1"/>
       <c r="S119" s="1"/>
     </row>
-    <row r="120">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -3657,7 +3674,7 @@
       <c r="R120" s="1"/>
       <c r="S120" s="1"/>
     </row>
-    <row r="121">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -3678,7 +3695,7 @@
       <c r="R121" s="1"/>
       <c r="S121" s="1"/>
     </row>
-    <row r="122">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -3699,7 +3716,7 @@
       <c r="R122" s="1"/>
       <c r="S122" s="1"/>
     </row>
-    <row r="123">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -3720,7 +3737,7 @@
       <c r="R123" s="1"/>
       <c r="S123" s="1"/>
     </row>
-    <row r="124">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -3741,7 +3758,7 @@
       <c r="R124" s="1"/>
       <c r="S124" s="1"/>
     </row>
-    <row r="125">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -3762,7 +3779,7 @@
       <c r="R125" s="1"/>
       <c r="S125" s="1"/>
     </row>
-    <row r="126">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -3783,7 +3800,7 @@
       <c r="R126" s="1"/>
       <c r="S126" s="1"/>
     </row>
-    <row r="127">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -3804,7 +3821,7 @@
       <c r="R127" s="1"/>
       <c r="S127" s="1"/>
     </row>
-    <row r="128">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -3825,7 +3842,7 @@
       <c r="R128" s="1"/>
       <c r="S128" s="1"/>
     </row>
-    <row r="129">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -3846,7 +3863,7 @@
       <c r="R129" s="1"/>
       <c r="S129" s="1"/>
     </row>
-    <row r="130">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -3867,7 +3884,7 @@
       <c r="R130" s="1"/>
       <c r="S130" s="1"/>
     </row>
-    <row r="131">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -3888,7 +3905,7 @@
       <c r="R131" s="1"/>
       <c r="S131" s="1"/>
     </row>
-    <row r="132">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -3909,7 +3926,7 @@
       <c r="R132" s="1"/>
       <c r="S132" s="1"/>
     </row>
-    <row r="133">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -3930,7 +3947,7 @@
       <c r="R133" s="1"/>
       <c r="S133" s="1"/>
     </row>
-    <row r="134">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -3951,7 +3968,7 @@
       <c r="R134" s="1"/>
       <c r="S134" s="1"/>
     </row>
-    <row r="135">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -3972,7 +3989,7 @@
       <c r="R135" s="1"/>
       <c r="S135" s="1"/>
     </row>
-    <row r="136">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -3993,7 +4010,7 @@
       <c r="R136" s="1"/>
       <c r="S136" s="1"/>
     </row>
-    <row r="137">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -4014,7 +4031,7 @@
       <c r="R137" s="1"/>
       <c r="S137" s="1"/>
     </row>
-    <row r="138">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -4035,7 +4052,7 @@
       <c r="R138" s="1"/>
       <c r="S138" s="1"/>
     </row>
-    <row r="139">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -4056,7 +4073,7 @@
       <c r="R139" s="1"/>
       <c r="S139" s="1"/>
     </row>
-    <row r="140">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -4077,7 +4094,7 @@
       <c r="R140" s="1"/>
       <c r="S140" s="1"/>
     </row>
-    <row r="141">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -4098,7 +4115,7 @@
       <c r="R141" s="1"/>
       <c r="S141" s="1"/>
     </row>
-    <row r="142">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -4119,7 +4136,7 @@
       <c r="R142" s="1"/>
       <c r="S142" s="1"/>
     </row>
-    <row r="143">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -4140,7 +4157,7 @@
       <c r="R143" s="1"/>
       <c r="S143" s="1"/>
     </row>
-    <row r="144">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -4161,7 +4178,7 @@
       <c r="R144" s="1"/>
       <c r="S144" s="1"/>
     </row>
-    <row r="145">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -4182,7 +4199,7 @@
       <c r="R145" s="1"/>
       <c r="S145" s="1"/>
     </row>
-    <row r="146">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -4203,7 +4220,7 @@
       <c r="R146" s="1"/>
       <c r="S146" s="1"/>
     </row>
-    <row r="147">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -4224,7 +4241,7 @@
       <c r="R147" s="1"/>
       <c r="S147" s="1"/>
     </row>
-    <row r="148">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -4245,7 +4262,7 @@
       <c r="R148" s="1"/>
       <c r="S148" s="1"/>
     </row>
-    <row r="149">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -4266,7 +4283,7 @@
       <c r="R149" s="1"/>
       <c r="S149" s="1"/>
     </row>
-    <row r="150">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -4287,7 +4304,7 @@
       <c r="R150" s="1"/>
       <c r="S150" s="1"/>
     </row>
-    <row r="151">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -4308,7 +4325,7 @@
       <c r="R151" s="1"/>
       <c r="S151" s="1"/>
     </row>
-    <row r="152">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -4329,7 +4346,7 @@
       <c r="R152" s="1"/>
       <c r="S152" s="1"/>
     </row>
-    <row r="153">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -4350,7 +4367,7 @@
       <c r="R153" s="1"/>
       <c r="S153" s="1"/>
     </row>
-    <row r="154">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -4371,7 +4388,7 @@
       <c r="R154" s="1"/>
       <c r="S154" s="1"/>
     </row>
-    <row r="155">
+    <row r="155" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -4392,7 +4409,7 @@
       <c r="R155" s="1"/>
       <c r="S155" s="1"/>
     </row>
-    <row r="156">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -4413,7 +4430,7 @@
       <c r="R156" s="1"/>
       <c r="S156" s="1"/>
     </row>
-    <row r="157">
+    <row r="157" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -4434,7 +4451,7 @@
       <c r="R157" s="1"/>
       <c r="S157" s="1"/>
     </row>
-    <row r="158">
+    <row r="158" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -4455,7 +4472,7 @@
       <c r="R158" s="1"/>
       <c r="S158" s="1"/>
     </row>
-    <row r="159">
+    <row r="159" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
@@ -4476,7 +4493,7 @@
       <c r="R159" s="1"/>
       <c r="S159" s="1"/>
     </row>
-    <row r="160">
+    <row r="160" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -4497,7 +4514,7 @@
       <c r="R160" s="1"/>
       <c r="S160" s="1"/>
     </row>
-    <row r="161">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
@@ -4518,7 +4535,7 @@
       <c r="R161" s="1"/>
       <c r="S161" s="1"/>
     </row>
-    <row r="162">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -4539,7 +4556,7 @@
       <c r="R162" s="1"/>
       <c r="S162" s="1"/>
     </row>
-    <row r="163">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
@@ -4560,7 +4577,7 @@
       <c r="R163" s="1"/>
       <c r="S163" s="1"/>
     </row>
-    <row r="164">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -4581,7 +4598,7 @@
       <c r="R164" s="1"/>
       <c r="S164" s="1"/>
     </row>
-    <row r="165">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -4602,7 +4619,7 @@
       <c r="R165" s="1"/>
       <c r="S165" s="1"/>
     </row>
-    <row r="166">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -4623,7 +4640,7 @@
       <c r="R166" s="1"/>
       <c r="S166" s="1"/>
     </row>
-    <row r="167">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -4644,7 +4661,7 @@
       <c r="R167" s="1"/>
       <c r="S167" s="1"/>
     </row>
-    <row r="168">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -4665,7 +4682,7 @@
       <c r="R168" s="1"/>
       <c r="S168" s="1"/>
     </row>
-    <row r="169">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -4686,7 +4703,7 @@
       <c r="R169" s="1"/>
       <c r="S169" s="1"/>
     </row>
-    <row r="170">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
@@ -4707,7 +4724,7 @@
       <c r="R170" s="1"/>
       <c r="S170" s="1"/>
     </row>
-    <row r="171">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
@@ -4728,7 +4745,7 @@
       <c r="R171" s="1"/>
       <c r="S171" s="1"/>
     </row>
-    <row r="172">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
@@ -4749,7 +4766,7 @@
       <c r="R172" s="1"/>
       <c r="S172" s="1"/>
     </row>
-    <row r="173">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
@@ -4770,7 +4787,7 @@
       <c r="R173" s="1"/>
       <c r="S173" s="1"/>
     </row>
-    <row r="174">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -4791,7 +4808,7 @@
       <c r="R174" s="1"/>
       <c r="S174" s="1"/>
     </row>
-    <row r="175">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
@@ -4812,7 +4829,7 @@
       <c r="R175" s="1"/>
       <c r="S175" s="1"/>
     </row>
-    <row r="176">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -4833,7 +4850,7 @@
       <c r="R176" s="1"/>
       <c r="S176" s="1"/>
     </row>
-    <row r="177">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A177" s="1"/>
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
@@ -4854,7 +4871,7 @@
       <c r="R177" s="1"/>
       <c r="S177" s="1"/>
     </row>
-    <row r="178">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -4875,7 +4892,7 @@
       <c r="R178" s="1"/>
       <c r="S178" s="1"/>
     </row>
-    <row r="179">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A179" s="1"/>
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
@@ -4896,7 +4913,7 @@
       <c r="R179" s="1"/>
       <c r="S179" s="1"/>
     </row>
-    <row r="180">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -4917,7 +4934,7 @@
       <c r="R180" s="1"/>
       <c r="S180" s="1"/>
     </row>
-    <row r="181">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A181" s="1"/>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
@@ -4938,7 +4955,7 @@
       <c r="R181" s="1"/>
       <c r="S181" s="1"/>
     </row>
-    <row r="182">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -4959,7 +4976,7 @@
       <c r="R182" s="1"/>
       <c r="S182" s="1"/>
     </row>
-    <row r="183">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A183" s="1"/>
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
@@ -4980,7 +4997,7 @@
       <c r="R183" s="1"/>
       <c r="S183" s="1"/>
     </row>
-    <row r="184">
+    <row r="184" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -5001,7 +5018,7 @@
       <c r="R184" s="1"/>
       <c r="S184" s="1"/>
     </row>
-    <row r="185">
+    <row r="185" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -5022,7 +5039,7 @@
       <c r="R185" s="1"/>
       <c r="S185" s="1"/>
     </row>
-    <row r="186">
+    <row r="186" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A186" s="1"/>
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
@@ -5043,7 +5060,7 @@
       <c r="R186" s="1"/>
       <c r="S186" s="1"/>
     </row>
-    <row r="187">
+    <row r="187" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A187" s="1"/>
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
@@ -5064,7 +5081,7 @@
       <c r="R187" s="1"/>
       <c r="S187" s="1"/>
     </row>
-    <row r="188">
+    <row r="188" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A188" s="1"/>
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
@@ -5085,7 +5102,7 @@
       <c r="R188" s="1"/>
       <c r="S188" s="1"/>
     </row>
-    <row r="189">
+    <row r="189" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
@@ -5106,7 +5123,7 @@
       <c r="R189" s="1"/>
       <c r="S189" s="1"/>
     </row>
-    <row r="190">
+    <row r="190" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A190" s="1"/>
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
@@ -5127,7 +5144,7 @@
       <c r="R190" s="1"/>
       <c r="S190" s="1"/>
     </row>
-    <row r="191">
+    <row r="191" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A191" s="1"/>
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
@@ -5148,7 +5165,7 @@
       <c r="R191" s="1"/>
       <c r="S191" s="1"/>
     </row>
-    <row r="192">
+    <row r="192" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A192" s="1"/>
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>
@@ -5169,7 +5186,7 @@
       <c r="R192" s="1"/>
       <c r="S192" s="1"/>
     </row>
-    <row r="193">
+    <row r="193" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A193" s="1"/>
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
@@ -5190,7 +5207,7 @@
       <c r="R193" s="1"/>
       <c r="S193" s="1"/>
     </row>
-    <row r="194">
+    <row r="194" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A194" s="1"/>
       <c r="B194" s="1"/>
       <c r="C194" s="1"/>
@@ -5211,7 +5228,7 @@
       <c r="R194" s="1"/>
       <c r="S194" s="1"/>
     </row>
-    <row r="195">
+    <row r="195" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -5232,7 +5249,7 @@
       <c r="R195" s="1"/>
       <c r="S195" s="1"/>
     </row>
-    <row r="196">
+    <row r="196" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
@@ -5253,7 +5270,7 @@
       <c r="R196" s="1"/>
       <c r="S196" s="1"/>
     </row>
-    <row r="197">
+    <row r="197" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -5274,7 +5291,7 @@
       <c r="R197" s="1"/>
       <c r="S197" s="1"/>
     </row>
-    <row r="198">
+    <row r="198" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>
@@ -5295,7 +5312,7 @@
       <c r="R198" s="1"/>
       <c r="S198" s="1"/>
     </row>
-    <row r="199">
+    <row r="199" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -5316,7 +5333,7 @@
       <c r="R199" s="1"/>
       <c r="S199" s="1"/>
     </row>
-    <row r="200">
+    <row r="200" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A200" s="1"/>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -5337,7 +5354,7 @@
       <c r="R200" s="1"/>
       <c r="S200" s="1"/>
     </row>
-    <row r="201">
+    <row r="201" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -5358,7 +5375,7 @@
       <c r="R201" s="1"/>
       <c r="S201" s="1"/>
     </row>
-    <row r="202">
+    <row r="202" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
@@ -5379,7 +5396,7 @@
       <c r="R202" s="1"/>
       <c r="S202" s="1"/>
     </row>
-    <row r="203">
+    <row r="203" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -5400,7 +5417,7 @@
       <c r="R203" s="1"/>
       <c r="S203" s="1"/>
     </row>
-    <row r="204">
+    <row r="204" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A204" s="1"/>
       <c r="B204" s="1"/>
       <c r="C204" s="1"/>
@@ -5421,7 +5438,7 @@
       <c r="R204" s="1"/>
       <c r="S204" s="1"/>
     </row>
-    <row r="205">
+    <row r="205" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -5442,7 +5459,7 @@
       <c r="R205" s="1"/>
       <c r="S205" s="1"/>
     </row>
-    <row r="206">
+    <row r="206" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
       <c r="C206" s="1"/>
@@ -5463,7 +5480,7 @@
       <c r="R206" s="1"/>
       <c r="S206" s="1"/>
     </row>
-    <row r="207">
+    <row r="207" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -5484,7 +5501,7 @@
       <c r="R207" s="1"/>
       <c r="S207" s="1"/>
     </row>
-    <row r="208">
+    <row r="208" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A208" s="1"/>
       <c r="B208" s="1"/>
       <c r="C208" s="1"/>
@@ -5505,7 +5522,7 @@
       <c r="R208" s="1"/>
       <c r="S208" s="1"/>
     </row>
-    <row r="209">
+    <row r="209" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -5526,7 +5543,7 @@
       <c r="R209" s="1"/>
       <c r="S209" s="1"/>
     </row>
-    <row r="210">
+    <row r="210" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
       <c r="C210" s="1"/>
@@ -5547,7 +5564,7 @@
       <c r="R210" s="1"/>
       <c r="S210" s="1"/>
     </row>
-    <row r="211">
+    <row r="211" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -5568,7 +5585,7 @@
       <c r="R211" s="1"/>
       <c r="S211" s="1"/>
     </row>
-    <row r="212">
+    <row r="212" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
@@ -5589,7 +5606,7 @@
       <c r="R212" s="1"/>
       <c r="S212" s="1"/>
     </row>
-    <row r="213">
+    <row r="213" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
@@ -5610,7 +5627,7 @@
       <c r="R213" s="1"/>
       <c r="S213" s="1"/>
     </row>
-    <row r="214">
+    <row r="214" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
@@ -5631,7 +5648,7 @@
       <c r="R214" s="1"/>
       <c r="S214" s="1"/>
     </row>
-    <row r="215">
+    <row r="215" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A215" s="1"/>
       <c r="B215" s="1"/>
       <c r="C215" s="1"/>
@@ -5652,7 +5669,7 @@
       <c r="R215" s="1"/>
       <c r="S215" s="1"/>
     </row>
-    <row r="216">
+    <row r="216" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A216" s="1"/>
       <c r="B216" s="1"/>
       <c r="C216" s="1"/>
@@ -5674,8 +5691,8 @@
       <c r="S216" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S16"/>
+  <autoFilter ref="A1:S16" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>